<commit_message>
agregando ejemplos a archivo de importacion
agregando ejemplos a archivo de importacion de catalogo de cuentas
</commit_message>
<xml_diff>
--- a/Backend/public/docs/catalogo-cuentas-format.xlsx
+++ b/Backend/public/docs/catalogo-cuentas-format.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28822"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jesus Alvarado\Documents\GitHub\Smartyme\Backend\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2029DC8C-A8E7-4460-AD8B-7871835F4277}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{37CCFB4C-29B1-4199-B56B-4241A011612B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2DA6AB23-7482-45C0-AB0B-8E26DD2DF24D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
   <si>
     <t>codigo</t>
   </si>
@@ -50,23 +50,80 @@
     <t>id_cuenta_padre</t>
   </si>
   <si>
+    <t>acepta_datos</t>
+  </si>
+  <si>
     <t>rubro</t>
   </si>
   <si>
     <t>nivel</t>
   </si>
   <si>
-    <t>acepta_datos</t>
-  </si>
-  <si>
     <t>saldo</t>
+  </si>
+  <si>
+    <t>Activo</t>
+  </si>
+  <si>
+    <t>Deudor</t>
+  </si>
+  <si>
+    <t>NO</t>
+  </si>
+  <si>
+    <t>Activos</t>
+  </si>
+  <si>
+    <t>Activos Corrientes</t>
+  </si>
+  <si>
+    <t>Efectivo y equivalentes</t>
+  </si>
+  <si>
+    <t>Efectivo en caja</t>
+  </si>
+  <si>
+    <t>Caja General</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Caja Chica</t>
+  </si>
+  <si>
+    <t>Efectivo en Bancos</t>
+  </si>
+  <si>
+    <t>Acreedor</t>
+  </si>
+  <si>
+    <t>Cuentas Corrientes</t>
+  </si>
+  <si>
+    <t>Banco xxx</t>
+  </si>
+  <si>
+    <t>Cuentas de Ahorro</t>
+  </si>
+  <si>
+    <t>Depósito a plazos</t>
+  </si>
+  <si>
+    <t>Mario de Jesus Peña</t>
+  </si>
+  <si>
+    <t>Cuentas y documentos por pagar</t>
+  </si>
+  <si>
+    <t>Pasivos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -446,19 +503,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A964E4CA-8297-42A2-A34B-1B7B384864B8}">
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="13.109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="47.109375" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.109375" customWidth="1"/>
-    <col min="7" max="7" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="47.140625" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.140625" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" s="1" customFormat="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -472,16 +529,347 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="15">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15">
+      <c r="A3" s="3">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="3">
+        <v>1101</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="3">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>16789</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="3">
+        <v>110101</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="3">
+        <v>1101</v>
+      </c>
+      <c r="E5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="3">
+        <v>11010101</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1698</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="3">
+        <v>11010102</v>
+      </c>
+      <c r="B7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="3">
+        <v>11010101</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="3">
+        <v>110102</v>
+      </c>
+      <c r="B8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="3">
+        <v>11010102</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="3">
+        <v>11010201</v>
+      </c>
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3">
+        <v>110102</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="3">
+        <v>1101020101</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="3">
+        <v>11010202</v>
+      </c>
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="3">
+        <v>1101020101</v>
+      </c>
+      <c r="E11" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="3">
+        <v>11010203</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="3">
+        <v>11010202</v>
+      </c>
+      <c r="E12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="3">
+        <v>11010204</v>
+      </c>
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" s="3">
+        <v>11010203</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="3">
+        <v>2102</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14">
+        <v>21</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14">
+        <v>2</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>